<commit_message>
Add YouTube banner, design docs, and archived MA/PhD page
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SVG-Logos/ICS-Graphics.xlsx
+++ b/SVG-Logos/ICS-Graphics.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/transferportal/Codex/1SharedResources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/transferportal/Github/ics-site/SVG-Logos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CD181C3-3E22-0340-BEBC-3125CB8A689E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE058BAB-C2F4-534C-9F0C-247BC34E4A4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1260" yWindow="600" windowWidth="29040" windowHeight="15720" xr2:uid="{7DA80EA3-7D56-4434-875F-54D99AFFE672}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>Graphic-Description</t>
   </si>
@@ -77,12 +77,6 @@
     <t>https://files.constantcontact.com/0e42c4d3901/5bbacbb2-09f4-4a95-a683-81dd03eefc8b.png</t>
   </si>
   <si>
-    <t>DanBeerensSignature - white background</t>
-  </si>
-  <si>
-    <t>https://files.constantcontact.com/0e42c4d3901/2a63bb3d-eafe-4edb-8584-babfd145e2ff.png</t>
-  </si>
-  <si>
     <t>https://files.constantcontact.com/0e42c4d3901/b68077cf-4711-44db-9eb7-3da505175135.png</t>
   </si>
   <si>
@@ -123,12 +117,6 @@
   </si>
   <si>
     <t>Ron Headshot (nose is at top left rule of thirds intersection)</t>
-  </si>
-  <si>
-    <t>Beth Signature</t>
-  </si>
-  <si>
-    <t>https://files.constantcontact.com/0e42c4d3901/6ae72d3d-8ef2-4856-9414-5904741732d2.png</t>
   </si>
 </sst>
 </file>
@@ -507,7 +495,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{932CA012-2F82-4DF6-BCAF-2A8C643798D4}">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.1640625" customWidth="1"/>
@@ -586,16 +574,16 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="C6">
-        <v>742</v>
+        <v>1200</v>
       </c>
       <c r="D6">
-        <v>226</v>
+        <v>234</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -603,13 +591,13 @@
         <v>15</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C7">
         <v>1200</v>
       </c>
       <c r="D7">
-        <v>234</v>
+        <v>296</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -617,18 +605,18 @@
         <v>17</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C8">
-        <v>1200</v>
+        <v>834</v>
       </c>
       <c r="D8">
-        <v>296</v>
+        <v>835</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>21</v>
@@ -642,10 +630,10 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="C10">
         <v>834</v>
@@ -656,40 +644,18 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C11">
-        <v>834</v>
-      </c>
-      <c r="D11">
-        <v>835</v>
+      <c r="B11" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" t="s">
         <v>24</v>
-      </c>
-      <c r="B12" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>28</v>
-      </c>
-      <c r="B14" t="s">
-        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>